<commit_message>
Redacción de entregables sin avisos de ejemplo, simulador web completo con plumas corregidas y portería virtual en el sistema Python
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLZ2XuhTWTWujj27otXiLx
</commit_message>
<xml_diff>
--- a/docs/documentos/01 Cronograma de Actividades.xlsx
+++ b/docs/documentos/01 Cronograma de Actividades.xlsx
@@ -884,7 +884,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Caso del Cliente (ficticio) y definición VIS/VIP/No VIP</t>
+          <t>Caso del Cliente y definición VIS/VIP/No VIP</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Caso del Cliente (ficticio) y definición VIS/VIP/No VIP</t>
+          <t>Caso del Cliente y definición VIS/VIP/No VIP</t>
         </is>
       </c>
       <c r="C11" s="9" t="n">

</xml_diff>

<commit_message>
Página web como sitio de producto, bitácora pública y limpieza de información interna
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLZ2XuhTWTWujj27otXiLx
</commit_message>
<xml_diff>
--- a/docs/documentos/01 Cronograma de Actividades.xlsx
+++ b/docs/documentos/01 Cronograma de Actividades.xlsx
@@ -925,7 +925,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Por asignar (acordar con el docente)</t>
+          <t>Por asignar</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
@@ -961,7 +961,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Por asignar (acordar con el docente)</t>
+          <t>Por asignar</t>
         </is>
       </c>
       <c r="D13" s="5" t="n">
@@ -997,7 +997,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Por asignar (acordar con el docente)</t>
+          <t>Por asignar</t>
         </is>
       </c>
       <c r="D14" s="5" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Por asignar (acordar con el docente)</t>
+          <t>Por asignar</t>
         </is>
       </c>
       <c r="D15" s="5" t="n">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Por asignar (acordar con el docente)</t>
+          <t>Por asignar</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Por asignar (acordar con el docente)</t>
+          <t>Por asignar</t>
         </is>
       </c>
       <c r="D25" s="5" t="n">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Por asignar (acordar con el docente)</t>
+          <t>Por asignar</t>
         </is>
       </c>
       <c r="D26" s="5" t="n">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Por asignar (acordar con el docente)</t>
+          <t>Por asignar</t>
         </is>
       </c>
       <c r="D27" s="5" t="n">
@@ -1501,7 +1501,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Por asignar (acordar con el docente)</t>
+          <t>Por asignar</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Por asignar (acordar con el docente)</t>
+          <t>Por asignar</t>
         </is>
       </c>
       <c r="D29" s="5" t="n">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Por asignar (acordar con el docente)</t>
+          <t>Por asignar</t>
         </is>
       </c>
       <c r="D36" s="5" t="n">
@@ -1851,7 +1851,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Notas: (1) Ningún estado es «Hecho»: solo el docente puede marcarlo. (2) Los responsables de actividades sin asignar se acuerdan con el docente. (3) Fechas propuestas, no acordadas.</t>
+          <t>Notas: (1) Ningún estado es «Hecho»: solo el docente puede marcarlo. (2) Los responsables de actividades sin asignar se definen en el equipo. (3) Fechas propuestas, no acordadas.</t>
         </is>
       </c>
     </row>

</xml_diff>